<commit_message>
modified:   .DS_Store 	modified:   README.md 	modified:   data/external/.DS_Store 	modified:   data/processed/categories_msw_composition.xlsx 	new file:   data/processed/msw_wf_composition.csv 	new file:   data/processed/msw_wf_composition_percent.csv 	new file:   data/processed/msw_wf_composition_v2.csv 	new file:   data/processed/msw_wf_composition_v3.csv 	new file:   data/processed/msw_wf_composition_v4.csv 	modified:   model/1.3 msw_composition_data.ipynb 	modified:   model/3.1 plot.ipynb 	modified:   model/3.2 plot_final.ipynb 	modified:   model/plot.py 	modified:   plots/.DS_Store 	new file:   plots/plot1/all_totals.png 	new file:   plots/plot1/tot_exc_min_weee.png     new file:   plots/plot1/total_exc_min_weee_sludge_chem.png 	new file:   plots/plot1/total_exc_minetc_sorting residue.png
</commit_message>
<xml_diff>
--- a/data/processed/categories_msw_composition.xlsx
+++ b/data/processed/categories_msw_composition.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marriyapillais/Desktop/msw_model/MSWI_Ash/data/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7C09696-3B98-AF4C-A749-49B4A295AC16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{442A66D1-CDFF-EB47-9ADD-EF32AE53276B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="660" windowWidth="24980" windowHeight="16720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2540" yWindow="660" windowWidth="24980" windowHeight="16660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="124">
   <si>
     <t>Waste categories</t>
   </si>
@@ -374,6 +375,24 @@
   </si>
   <si>
     <t>Disaggregated categories</t>
+  </si>
+  <si>
+    <t>weee + batt + vehicles</t>
+  </si>
+  <si>
+    <t>chemical and medical</t>
+  </si>
+  <si>
+    <t>metal</t>
+  </si>
+  <si>
+    <t>common sludges</t>
+  </si>
+  <si>
+    <t>mineral waste</t>
+  </si>
+  <si>
+    <t>organic waste</t>
   </si>
 </sst>
 </file>
@@ -1324,6 +1343,579 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1593CE5-D492-C242-B23B-3E6A6C4A7B0C}">
+  <dimension ref="A1:E50"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="60.5" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="4" max="4" width="25.5" customWidth="1"/>
+    <col min="5" max="5" width="36.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" t="s">
+        <v>39</v>
+      </c>
+      <c r="E20" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" t="s">
+        <v>41</v>
+      </c>
+      <c r="E21" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" t="s">
+        <v>43</v>
+      </c>
+      <c r="E22" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" t="s">
+        <v>45</v>
+      </c>
+      <c r="E23" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" t="s">
+        <v>47</v>
+      </c>
+      <c r="C24" t="s">
+        <v>47</v>
+      </c>
+      <c r="D24" t="s">
+        <v>47</v>
+      </c>
+      <c r="E24" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26" t="s">
+        <v>51</v>
+      </c>
+      <c r="E26" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>54</v>
+      </c>
+      <c r="B28" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>56</v>
+      </c>
+      <c r="B29" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>60</v>
+      </c>
+      <c r="B31" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>62</v>
+      </c>
+      <c r="B32" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" t="s">
+        <v>65</v>
+      </c>
+      <c r="D33" t="s">
+        <v>65</v>
+      </c>
+      <c r="E33" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>66</v>
+      </c>
+      <c r="B34" t="s">
+        <v>67</v>
+      </c>
+      <c r="C34" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>68</v>
+      </c>
+      <c r="B35" t="s">
+        <v>69</v>
+      </c>
+      <c r="C35" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36" t="s">
+        <v>71</v>
+      </c>
+      <c r="C36" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>72</v>
+      </c>
+      <c r="B37" t="s">
+        <v>73</v>
+      </c>
+      <c r="D37" t="s">
+        <v>73</v>
+      </c>
+      <c r="E37" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>74</v>
+      </c>
+      <c r="B38" t="s">
+        <v>75</v>
+      </c>
+      <c r="D38" t="s">
+        <v>75</v>
+      </c>
+      <c r="E38" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>76</v>
+      </c>
+      <c r="B39" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>80</v>
+      </c>
+      <c r="B41" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>82</v>
+      </c>
+      <c r="B42" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>84</v>
+      </c>
+      <c r="B43" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>86</v>
+      </c>
+      <c r="B44" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>88</v>
+      </c>
+      <c r="B45" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>90</v>
+      </c>
+      <c r="B46" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>92</v>
+      </c>
+      <c r="B47" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>94</v>
+      </c>
+      <c r="B48" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>96</v>
+      </c>
+      <c r="B49" t="s">
+        <v>97</v>
+      </c>
+      <c r="C49" t="s">
+        <v>97</v>
+      </c>
+      <c r="D49" t="s">
+        <v>97</v>
+      </c>
+      <c r="E49" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>98</v>
+      </c>
+      <c r="B50" t="s">
+        <v>99</v>
+      </c>
+      <c r="C50" t="s">
+        <v>99</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{d465f887-04a9-4c17-8b62-103eddccf68b}" enabled="1" method="Standard" siteId="{ca2a7f76-dbd7-4ec0-9108-6b3d524fb7c8}" contentBits="0" removed="0"/>

</xml_diff>